<commit_message>
Case, Nested Case, Create statement
</commit_message>
<xml_diff>
--- a/Excel/Dynamic_Dashboard/Excel+Dashboard+2 (4).xlsx
+++ b/Excel/Dynamic_Dashboard/Excel+Dashboard+2 (4).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DC_DDS_01\Excel\Dynamic_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCACB111-F948-40E4-BDD5-AE46771A3608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B0D2DA-322B-4754-A918-FCE24B2B0946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="53">
   <si>
     <t>ProductionID</t>
   </si>
@@ -183,9 +183,6 @@
     <t>Sum of UnitsProduced</t>
   </si>
   <si>
-    <t>2023</t>
-  </si>
-  <si>
     <t>Sep</t>
   </si>
   <si>
@@ -229,6 +226,9 @@
   </si>
   <si>
     <t>Production Dashboard</t>
+  </si>
+  <si>
+    <t>2024</t>
   </si>
 </sst>
 </file>
@@ -314,6 +314,7 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -326,13 +327,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="7">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     </dxf>
@@ -619,19 +634,13 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 1'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 1'!$A$4:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Automobiles</c:v>
+                  <c:v>Furniture</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Electronics</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Furniture</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -639,21 +648,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 1'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 1'!$B$4:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>142768</c:v>
+                  <c:v>7125</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>679</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>90859</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>178302</c:v>
+                  <c:v>16864</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1154,59 +1157,23 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 2'!$A$4:$A$11</c:f>
+              <c:f>'Pivot 2'!$A$4:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Jane Smith</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Laura Black</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>David White</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Mike Brown</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>Nancy Grey</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Andrew Blue</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>John Doe</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 2'!$B$4:$B$11</c:f>
+              <c:f>'Pivot 2'!$B$4:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="1">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1651,23 +1618,20 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'Pivot 3'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 3'!$A$4:$A$7</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>Oct</c:v>
+                    <c:v>Feb</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>Nov</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Dec</c:v>
+                    <c:v>Mar</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>2023</c:v>
+                    <c:v>2024</c:v>
                   </c:pt>
                 </c:lvl>
               </c:multiLvlStrCache>
@@ -1675,18 +1639,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 3'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 3'!$B$4:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1143</c:v>
+                  <c:v>318</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1840</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>959</c:v>
+                  <c:v>218</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2187,7 +2148,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="FFCCCC"/>
+                <a:srgbClr val="FFCC99"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -2212,7 +2173,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCFFCC"/>
+                <a:srgbClr val="CCCCFF"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -2237,7 +2198,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="FFCC99"/>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -2262,7 +2223,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCCCFF"/>
+                <a:schemeClr val="accent4"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -2337,19 +2298,13 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 4'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 4'!$A$4:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Automobiles</c:v>
+                  <c:v>Furniture</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Electronics</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Furniture</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -2357,21 +2312,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 4'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 4'!$B$4:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>116.07783789987161</c:v>
+                  <c:v>32.683486238532112</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2117263843648209</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>82.9945217959296</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>178.306304928782</c:v>
+                  <c:v>53.031446540880502</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2875,19 +2824,13 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 1'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 1'!$A$4:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Automobiles</c:v>
+                  <c:v>Furniture</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Electronics</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Furniture</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -2895,21 +2838,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 1'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 1'!$B$4:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>142768</c:v>
+                  <c:v>7125</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>679</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>90859</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>178302</c:v>
+                  <c:v>16864</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3576,59 +3513,23 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 2'!$A$4:$A$11</c:f>
+              <c:f>'Pivot 2'!$A$4:$A$5</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Jane Smith</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Laura Black</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>David White</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Mike Brown</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>Nancy Grey</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Andrew Blue</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>John Doe</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 2'!$B$4:$B$11</c:f>
+              <c:f>'Pivot 2'!$B$4:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="1">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4211,23 +4112,20 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'Pivot 3'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 3'!$A$4:$A$7</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>Oct</c:v>
+                    <c:v>Feb</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>Nov</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Dec</c:v>
+                    <c:v>Mar</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>2023</c:v>
+                    <c:v>2024</c:v>
                   </c:pt>
                 </c:lvl>
               </c:multiLvlStrCache>
@@ -4235,18 +4133,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 3'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 3'!$B$4:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1143</c:v>
+                  <c:v>318</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1840</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>959</c:v>
+                  <c:v>218</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5021,7 +4916,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="FFCCCC"/>
+                <a:srgbClr val="FFCC99"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -5046,7 +4941,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCFFCC"/>
+                <a:srgbClr val="CCCCFF"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -5071,7 +4966,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="FFCC99"/>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -5096,7 +4991,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCCCFF"/>
+                <a:schemeClr val="accent4"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -5171,19 +5066,13 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 4'!$A$4:$A$8</c:f>
+              <c:f>'Pivot 4'!$A$4:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Automobiles</c:v>
+                  <c:v>Furniture</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Electronics</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Furniture</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -5191,21 +5080,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 4'!$B$4:$B$8</c:f>
+              <c:f>'Pivot 4'!$B$4:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>116.07783789987161</c:v>
+                  <c:v>32.683486238532112</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2117263843648209</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>82.9945217959296</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>178.306304928782</c:v>
+                  <c:v>53.031446540880502</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13325,7 +13208,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B4A05C44-8E02-4C0B-897E-E209559CB89E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13434,10 +13317,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item x="3"/>
+        <item h="1" x="3"/>
         <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
+        <item h="1" x="0"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13455,8 +13338,8 @@
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item t="default"/>
       </items>
@@ -13464,9 +13347,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="2"/>
-        <item x="1"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13493,10 +13376,10 @@
     <pivotField showAll="0">
       <items count="7">
         <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item h="1" x="3"/>
-        <item x="4"/>
+        <item h="1" x="4"/>
         <item h="1" x="5"/>
         <item t="default"/>
       </items>
@@ -13514,13 +13397,7 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
+  <rowItems count="3">
     <i>
       <x v="2"/>
     </i>
@@ -13538,7 +13415,7 @@
     <dataField name="Sum of TotalCost" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="1">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -13576,7 +13453,7 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4EE43A99-DA69-49C7-9999-13295477D628}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A3:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField dataField="1" showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13685,10 +13562,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item x="3"/>
+        <item h="1" x="3"/>
         <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
+        <item h="1" x="0"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13721,8 +13598,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item t="default"/>
       </items>
@@ -13730,9 +13607,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="2"/>
-        <item x="1"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13759,10 +13636,10 @@
     <pivotField showAll="0">
       <items count="7">
         <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item h="1" x="3"/>
-        <item x="4"/>
+        <item h="1" x="4"/>
         <item h="1" x="5"/>
         <item t="default"/>
       </items>
@@ -13780,27 +13657,9 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
+  <rowItems count="2">
     <i>
       <x v="8"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="5"/>
     </i>
     <i t="grand">
       <x/>
@@ -13846,7 +13705,7 @@
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8D064263-4D1C-40D7-BF76-F231D23CFDA0}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13955,10 +13814,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item x="3"/>
+        <item h="1" x="3"/>
         <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
+        <item h="1" x="0"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13968,8 +13827,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item t="default"/>
       </items>
@@ -13977,9 +13836,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="2"/>
-        <item x="1"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -14006,10 +13865,10 @@
     <pivotField showAll="0">
       <items count="7">
         <item h="1" sd="0" x="0"/>
-        <item h="1" sd="0" x="1"/>
+        <item sd="0" x="1"/>
         <item h="1" sd="0" x="2"/>
         <item h="1" sd="0" x="3"/>
-        <item sd="0" x="4"/>
+        <item h="1" sd="0" x="4"/>
         <item h="1" sd="0" x="5"/>
         <item t="default"/>
       </items>
@@ -14028,18 +13887,15 @@
     <field x="13"/>
     <field x="11"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="4">
     <i>
-      <x v="1"/>
+      <x v="2"/>
     </i>
     <i r="1">
-      <x v="10"/>
+      <x v="2"/>
     </i>
     <i r="1">
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -14085,7 +13941,7 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{87307F0E-6F33-40F7-A92A-4E423868BB78}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -14194,10 +14050,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item x="3"/>
+        <item h="1" x="3"/>
         <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
+        <item h="1" x="0"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -14215,8 +14071,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
-        <item h="1" x="1"/>
+        <item h="1" x="0"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item t="default"/>
       </items>
@@ -14224,9 +14080,9 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="2"/>
-        <item x="1"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -14235,10 +14091,10 @@
     <pivotField showAll="0" defaultSubtotal="0">
       <items count="6">
         <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item h="1" x="2"/>
         <item h="1" x="3"/>
-        <item x="4"/>
+        <item h="1" x="4"/>
         <item h="1" x="5"/>
       </items>
     </pivotField>
@@ -14254,13 +14110,7 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
+  <rowItems count="3">
     <i>
       <x v="2"/>
     </i>
@@ -14569,7 +14419,7 @@
     <dataField name="Sum of TotalCost" fld="6" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="0">
+    <format dxfId="5">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14850,10 +14700,10 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="4">
-        <i x="3" s="1"/>
+        <i x="3"/>
         <i x="2" s="1"/>
-        <i x="0" s="1"/>
-        <i x="1" s="1"/>
+        <i x="0"/>
+        <i x="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -14871,9 +14721,9 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="3">
-        <i x="0" s="1"/>
-        <i x="1"/>
-        <i x="2"/>
+        <i x="1" s="1"/>
+        <i x="0" nd="1"/>
+        <i x="2" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -14891,9 +14741,9 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="3">
-        <i x="0" s="1"/>
+        <i x="0"/>
         <i x="2" s="1"/>
-        <i x="1" s="1"/>
+        <i x="1"/>
       </items>
     </tabular>
   </data>
@@ -14911,10 +14761,10 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="6">
-        <i x="1"/>
+        <i x="1" s="1"/>
         <i x="2"/>
         <i x="3"/>
-        <i x="4" s="1"/>
+        <i x="4"/>
         <i x="0" nd="1"/>
         <i x="5" nd="1"/>
       </items>
@@ -15258,7 +15108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC7590B-59C1-4780-B184-059AA2CBDAFA}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15275,42 +15125,26 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B4" s="5">
-        <v>142768</v>
+        <v>7125</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B5" s="5">
-        <v>679</v>
+        <v>16864</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5">
-        <v>90859</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="5">
-        <v>178302</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="5">
-        <v>412608</v>
+        <v>23989</v>
       </c>
     </row>
   </sheetData>
@@ -15321,7 +15155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F52287D6-AC2A-495B-8F15-E05B7FBCCBFF}">
-  <dimension ref="A3:B11"/>
+  <dimension ref="A3:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15338,66 +15172,18 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B4" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B5" s="13">
         <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="13">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -15408,7 +15194,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F3A811-0A1A-4FEF-9853-B1FFC57DE7E8}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15425,42 +15211,34 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="B4" s="13">
-        <v>3942</v>
+        <v>536</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B5" s="13">
-        <v>1143</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B6" s="13">
-        <v>1840</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>41</v>
+      <c r="A7" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="B7" s="13">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="13">
-        <v>3942</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>
@@ -15472,7 +15250,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31661C08-08AE-40BA-AF39-38EBBD305E22}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15484,47 +15262,31 @@
         <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B4" s="13">
-        <v>116.07783789987161</v>
+        <v>32.683486238532112</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B5" s="13">
-        <v>2.2117263843648209</v>
+        <v>53.031446540880502</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B6" s="13">
-        <v>82.9945217959296</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="13">
-        <v>178.306304928782</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="13">
-        <v>114.04471030444071</v>
+        <v>42.857466389706303</v>
       </c>
     </row>
   </sheetData>
@@ -15539,110 +15301,110 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
+      <c r="A1" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="9"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
-      <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -15733,70 +15495,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
+      <c r="A1" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="11"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
@@ -15808,7 +15570,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9">
         <v>3026</v>
@@ -15816,7 +15578,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10">
         <v>4127</v>
@@ -15824,7 +15586,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B11">
         <v>3875</v>
@@ -15832,7 +15594,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B12">
         <v>1528</v>
@@ -15840,7 +15602,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B13">
         <v>1684</v>
@@ -15848,7 +15610,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14">
         <v>3537</v>
@@ -15856,7 +15618,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B15">
         <v>1536</v>
@@ -15864,7 +15626,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B16">
         <v>2864</v>
@@ -15872,7 +15634,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17">
         <v>2150</v>
@@ -15880,7 +15642,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18">
         <v>3103</v>
@@ -15888,7 +15650,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19">
         <v>4803</v>
@@ -15896,7 +15658,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20">
         <v>2494</v>
@@ -15945,37 +15707,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="8" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Constraints in sql and order of execution
</commit_message>
<xml_diff>
--- a/Excel/Dynamic_Dashboard/Excel+Dashboard+2 (4).xlsx
+++ b/Excel/Dynamic_Dashboard/Excel+Dashboard+2 (4).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DC_DDS_01\Excel\Dynamic_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B0D2DA-322B-4754-A918-FCE24B2B0946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62948D3-6880-43A9-AA17-376A8D91C979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot 1" sheetId="8" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="56">
   <si>
     <t>ProductionID</t>
   </si>
@@ -230,6 +230,15 @@
   <si>
     <t>2024</t>
   </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Product Type</t>
+  </si>
 </sst>
 </file>
 
@@ -332,13 +341,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     </dxf>
@@ -634,13 +637,19 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 1'!$A$4:$A$6</c:f>
+              <c:f>'Pivot 1'!$A$4:$A$8</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Automobiles</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Electronics</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Furniture</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -648,15 +657,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 1'!$B$4:$B$6</c:f>
+              <c:f>'Pivot 1'!$B$4:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>7125</c:v>
+                  <c:v>800360</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16864</c:v>
+                  <c:v>341435</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>446302</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>561014</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1157,23 +1172,77 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 2'!$A$4:$A$5</c:f>
+              <c:f>'Pivot 2'!$A$4:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>Nancy Grey</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Jane Smith</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Laura Black</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>John Doe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Andrew Blue</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Mike Brown</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Emily Davis</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>David White</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sarah Lee</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Chris Green</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 2'!$B$4:$B$5</c:f>
+              <c:f>'Pivot 2'!$B$4:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1618,19 +1687,46 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'Pivot 3'!$A$4:$A$7</c:f>
+              <c:f>'Pivot 3'!$A$4:$A$16</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="10"/>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>Feb</c:v>
+                    <c:v>Sep</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>Mar</c:v>
+                    <c:v>Oct</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Nov</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Dec</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Apr</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>May</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Jun</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Jul</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Aug</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Sep</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
+                    <c:v>2023</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
                     <c:v>2024</c:v>
                   </c:pt>
                 </c:lvl>
@@ -1639,15 +1735,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 3'!$B$4:$B$7</c:f>
+              <c:f>'Pivot 3'!$B$4:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>318</c:v>
+                  <c:v>771</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>218</c:v>
+                  <c:v>3103</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4803</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2494</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1528</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1684</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3537</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1536</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2864</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1379</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2013,7 +2133,7 @@
         <c:idx val="1"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="CCCCFF"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -2032,7 +2152,7 @@
         <c:idx val="2"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="FFCCCC"/>
+            <a:srgbClr val="FFCC99"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -2051,7 +2171,7 @@
         <c:idx val="3"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="CCFFCC"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -2070,7 +2190,7 @@
         <c:idx val="4"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="FFCC99"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -2173,7 +2293,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCCCFF"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -2298,13 +2418,19 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 4'!$A$4:$A$6</c:f>
+              <c:f>'Pivot 4'!$A$4:$A$8</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Automobiles</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Electronics</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Furniture</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -2312,15 +2438,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 4'!$B$4:$B$6</c:f>
+              <c:f>'Pivot 4'!$B$4:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>32.683486238532112</c:v>
+                  <c:v>136.50595386143647</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>53.031446540880502</c:v>
+                  <c:v>106.84509125545883</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>157.61176084289789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>111.05339553555136</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2824,13 +2956,19 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 1'!$A$4:$A$6</c:f>
+              <c:f>'Pivot 1'!$A$4:$A$8</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Automobiles</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Electronics</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Furniture</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -2838,15 +2976,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 1'!$B$4:$B$6</c:f>
+              <c:f>'Pivot 1'!$B$4:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0_);_(* \(#,##0\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>7125</c:v>
+                  <c:v>800360</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16864</c:v>
+                  <c:v>341435</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>446302</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>561014</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3513,23 +3657,77 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 2'!$A$4:$A$5</c:f>
+              <c:f>'Pivot 2'!$A$4:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>Nancy Grey</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Jane Smith</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Laura Black</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>John Doe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Andrew Blue</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Mike Brown</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Emily Davis</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>David White</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sarah Lee</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Chris Green</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 2'!$B$4:$B$5</c:f>
+              <c:f>'Pivot 2'!$B$4:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4112,19 +4310,46 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>'Pivot 3'!$A$4:$A$7</c:f>
+              <c:f>'Pivot 3'!$A$4:$A$16</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="10"/>
                 <c:lvl>
                   <c:pt idx="0">
-                    <c:v>Feb</c:v>
+                    <c:v>Sep</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>Mar</c:v>
+                    <c:v>Oct</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Nov</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Dec</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Apr</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>May</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Jun</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Jul</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Aug</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Sep</c:v>
                   </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
+                    <c:v>2023</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
                     <c:v>2024</c:v>
                   </c:pt>
                 </c:lvl>
@@ -4133,15 +4358,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 3'!$B$4:$B$7</c:f>
+              <c:f>'Pivot 3'!$B$4:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>318</c:v>
+                  <c:v>771</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>218</c:v>
+                  <c:v>3103</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4803</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2494</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1528</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1684</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3537</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1536</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2864</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1379</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4781,7 +5030,7 @@
         <c:idx val="11"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="FFCCCC"/>
+            <a:srgbClr val="FFCC99"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -4800,7 +5049,7 @@
         <c:idx val="12"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="CCFFCC"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -4819,7 +5068,7 @@
         <c:idx val="13"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="FFCC99"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -4838,7 +5087,7 @@
         <c:idx val="14"/>
         <c:spPr>
           <a:solidFill>
-            <a:srgbClr val="CCCCFF"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln w="25400">
             <a:solidFill>
@@ -4941,7 +5190,7 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="CCCCFF"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln w="25400">
                 <a:solidFill>
@@ -5066,13 +5315,19 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Pivot 4'!$A$4:$A$6</c:f>
+              <c:f>'Pivot 4'!$A$4:$A$8</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Automobiles</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Electronics</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Furniture</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>Machinery</c:v>
                 </c:pt>
               </c:strCache>
@@ -5080,15 +5335,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Pivot 4'!$B$4:$B$6</c:f>
+              <c:f>'Pivot 4'!$B$4:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="2"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>32.683486238532112</c:v>
+                  <c:v>136.50595386143647</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>53.031446540880502</c:v>
+                  <c:v>106.84509125545883</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>157.61176084289789</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>111.05339553555136</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10509,16 +10770,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>601980</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>11430</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>64770</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>144780</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>411480</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -13207,8 +13468,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B4A05C44-8E02-4C0B-897E-E209559CB89E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B4A05C44-8E02-4C0B-897E-E209559CB89E}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9" rowHeaderCaption="Product Type">
+  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13317,10 +13578,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item h="1" x="3"/>
+        <item x="3"/>
         <item x="2"/>
-        <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13338,18 +13599,18 @@
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="2"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13375,12 +13636,12 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="0"/>
-        <item x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item h="1" x="4"/>
-        <item h="1" x="5"/>
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13397,7 +13658,13 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
     <i>
       <x v="2"/>
     </i>
@@ -13412,10 +13679,10 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of TotalCost" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+    <dataField name="Total Cost" fld="6" baseField="4" baseItem="2" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="6">
+    <format dxfId="4">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -13453,7 +13720,7 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4EE43A99-DA69-49C7-9999-13295477D628}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField dataField="1" showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13562,10 +13829,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item h="1" x="3"/>
+        <item x="3"/>
         <item x="2"/>
-        <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13598,18 +13865,18 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="2"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13635,12 +13902,12 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="0"/>
-        <item x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item h="1" x="4"/>
-        <item h="1" x="5"/>
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13657,9 +13924,36 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="11">
     <i>
       <x v="8"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="1"/>
     </i>
     <i t="grand">
       <x/>
@@ -13705,7 +13999,7 @@
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8D064263-4D1C-40D7-BF76-F231D23CFDA0}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -13814,10 +14108,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item h="1" x="3"/>
+        <item x="3"/>
         <item x="2"/>
-        <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13827,18 +14121,18 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="2"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13864,12 +14158,12 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item h="1" sd="0" x="2"/>
-        <item h="1" sd="0" x="3"/>
-        <item h="1" sd="0" x="4"/>
-        <item h="1" sd="0" x="5"/>
+        <item sd="0" x="0"/>
+        <item h="1" sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13887,15 +14181,42 @@
     <field x="13"/>
     <field x="11"/>
   </rowFields>
-  <rowItems count="4">
+  <rowItems count="13">
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
     <i>
       <x v="2"/>
     </i>
     <i r="1">
-      <x v="2"/>
+      <x v="4"/>
     </i>
     <i r="1">
-      <x v="3"/>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
     </i>
     <i t="grand">
       <x/>
@@ -13941,7 +14262,7 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{87307F0E-6F33-40F7-A92A-4E423868BB78}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0">
@@ -14050,10 +14371,10 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="5">
-        <item h="1" x="3"/>
+        <item x="3"/>
         <item x="2"/>
-        <item h="1" x="0"/>
-        <item h="1" x="1"/>
+        <item x="0"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -14071,18 +14392,18 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="2"/>
-        <item h="1" x="1"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -14090,12 +14411,12 @@
     <pivotField showAll="0" defaultSubtotal="0"/>
     <pivotField showAll="0" defaultSubtotal="0">
       <items count="6">
-        <item h="1" x="0"/>
-        <item x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item h="1" x="4"/>
-        <item h="1" x="5"/>
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
       </items>
     </pivotField>
     <pivotField showAll="0" defaultSubtotal="0">
@@ -14110,7 +14431,13 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
     <i>
       <x v="2"/>
     </i>
@@ -14419,7 +14746,7 @@
     <dataField name="Sum of TotalCost" fld="6" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="5">
+    <format dxfId="3">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14700,10 +15027,10 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="4">
-        <i x="3"/>
+        <i x="3" s="1"/>
         <i x="2" s="1"/>
-        <i x="0"/>
-        <i x="1" nd="1"/>
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
       </items>
     </tabular>
   </data>
@@ -14721,9 +15048,9 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="3">
+        <i x="0" s="1"/>
         <i x="1" s="1"/>
-        <i x="0" nd="1"/>
-        <i x="2" nd="1"/>
+        <i x="2" s="1"/>
       </items>
     </tabular>
   </data>
@@ -14741,9 +15068,9 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="3">
-        <i x="0"/>
+        <i x="0" s="1"/>
         <i x="2" s="1"/>
-        <i x="1"/>
+        <i x="1" s="1"/>
       </items>
     </tabular>
   </data>
@@ -14761,12 +15088,12 @@
   <data>
     <tabular pivotCacheId="984892114">
       <items count="6">
-        <i x="1" s="1"/>
-        <i x="2"/>
-        <i x="3"/>
-        <i x="4"/>
-        <i x="0" nd="1"/>
-        <i x="5" nd="1"/>
+        <i x="1"/>
+        <i x="2" s="1"/>
+        <i x="3" s="1"/>
+        <i x="4" s="1"/>
+        <i x="0" s="1" nd="1"/>
+        <i x="5" s="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -14833,7 +15160,7 @@
   <slicer name="Region" xr10:uid="{9190ECA8-014F-4A4A-BEEC-CF300AC8D463}" cache="Slicer_Region" caption="Region" rowHeight="234950"/>
   <slicer name="Gender" xr10:uid="{BD07F61C-21A6-48A3-964E-72CBA6063C43}" cache="Slicer_Gender" caption="Gender" rowHeight="234950"/>
   <slicer name="Age Groups" xr10:uid="{8AFE9850-E87D-41A3-B551-3DF3ED874B5D}" cache="Slicer_Age_Groups" caption="Age Groups" rowHeight="234950"/>
-  <slicer name="Quarters (ProductionDate)" xr10:uid="{6323FAC9-8D51-47DE-8A27-A0AAC300EABF}" cache="Slicer_Quarters__ProductionDate" caption="Quarters (ProductionDate)" rowHeight="234950"/>
+  <slicer name="Quarters (ProductionDate)" xr10:uid="{6323FAC9-8D51-47DE-8A27-A0AAC300EABF}" cache="Slicer_Quarters__ProductionDate" caption="Quarters (ProductionDate)" startItem="1" rowHeight="234950"/>
 </slicers>
 </file>
 
@@ -15108,43 +15435,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC7590B-59C1-4780-B184-059AA2CBDAFA}">
-  <dimension ref="A3:B6"/>
+  <dimension ref="A3:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B4" s="5">
-        <v>7125</v>
+        <v>800360</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B5" s="5">
-        <v>16864</v>
+        <v>341435</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="5">
+        <v>446302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="5">
+        <v>561014</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="5">
-        <v>23989</v>
+      <c r="B8" s="5">
+        <v>2149111</v>
       </c>
     </row>
   </sheetData>
@@ -15155,7 +15498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F52287D6-AC2A-495B-8F15-E05B7FBCCBFF}">
-  <dimension ref="A3:B5"/>
+  <dimension ref="A3:B14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15175,15 +15518,87 @@
         <v>24</v>
       </c>
       <c r="B4" s="13">
-        <v>2</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="13">
-        <v>2</v>
+      <c r="B14" s="13">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -15194,7 +15609,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F3A811-0A1A-4FEF-9853-B1FFC57DE7E8}">
-  <dimension ref="A3:B7"/>
+  <dimension ref="A3:B16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15211,34 +15626,106 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B4" s="13">
-        <v>536</v>
+        <v>11171</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B5" s="13">
-        <v>318</v>
+        <v>771</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B6" s="13">
-        <v>218</v>
+        <v>3103</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="13">
+        <v>4803</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="13">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="13">
+        <v>12528</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="13">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="13">
+        <v>1684</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="13">
+        <v>3537</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="13">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="13">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="13">
+        <v>1379</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="13">
-        <v>536</v>
+      <c r="B16" s="13">
+        <v>23699</v>
       </c>
     </row>
   </sheetData>
@@ -15250,7 +15737,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31661C08-08AE-40BA-AF39-38EBBD305E22}">
-  <dimension ref="A3:B6"/>
+  <dimension ref="A3:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -15267,26 +15754,42 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B4" s="13">
-        <v>32.683486238532112</v>
+        <v>136.50595386143647</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B5" s="13">
-        <v>53.031446540880502</v>
+        <v>106.84509125545883</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="13">
+        <v>157.61176084289789</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="13">
+        <v>111.05339553555136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="13">
-        <v>42.857466389706303</v>
+      <c r="B8" s="13">
+        <v>128.2240455479031</v>
       </c>
     </row>
   </sheetData>

</xml_diff>